<commit_message>
gantt chart works for 'startline' and 'deadline'
</commit_message>
<xml_diff>
--- a/data/project_tasks.xlsx
+++ b/data/project_tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\WW FILES\Indie Project\gantt-plotter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E275D26C-4E60-45D0-95EE-DAF22B6E1724}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD14A596-B028-4A21-B9EE-42652B71123D}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="18084" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="18084" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -320,9 +320,6 @@
     <t>template_name</t>
   </si>
   <si>
-    <t>deadline</t>
-  </si>
-  <si>
     <t>buffer_days</t>
   </si>
   <si>
@@ -444,6 +441,9 @@
   </si>
   <si>
     <t xml:space="preserve">Presentasi FT </t>
+  </si>
+  <si>
+    <t>startline</t>
   </si>
 </sst>
 </file>
@@ -2598,7 +2598,7 @@
     <col min="4" max="4" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27.6">
+    <row r="1" spans="1:4">
       <c r="A1" s="8" t="s">
         <v>96</v>
       </c>
@@ -2606,18 +2606,18 @@
         <v>97</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C2" s="12">
         <v>46234</v>
@@ -2628,10 +2628,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" s="12">
         <v>46234</v>
@@ -2642,10 +2642,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C4" s="12">
         <v>46234</v>
@@ -2656,10 +2656,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="12">
         <v>46234</v>
@@ -2670,10 +2670,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="12">
         <v>46234</v>
@@ -2684,10 +2684,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" s="12">
         <v>46234</v>
@@ -2731,7 +2731,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2749,7 +2749,7 @@
         <v>2</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2769,7 +2769,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="27.6">
@@ -2789,7 +2789,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.6">
@@ -2809,7 +2809,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2829,7 +2829,7 @@
         <v>2</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2849,7 +2849,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="41.4">
@@ -2869,7 +2869,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.6">
@@ -2889,7 +2889,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2900,16 +2900,16 @@
         <v>4</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>122</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>123</v>
       </c>
       <c r="E10" s="9">
         <v>14</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2952,7 +2952,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="27.6">
@@ -2961,16 +2961,16 @@
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" s="9">
         <v>2</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2981,16 +2981,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -3001,16 +3001,16 @@
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E4" s="9">
         <v>1</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.6">
@@ -3021,16 +3021,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E5" s="9">
         <v>3</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.6">
@@ -3041,16 +3041,16 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E6" s="9">
         <v>2</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="41.4">
@@ -3061,16 +3061,16 @@
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E7" s="9">
         <v>2</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="41.4">
@@ -3081,16 +3081,16 @@
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E8" s="9">
         <v>2</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="41.4">
@@ -3101,16 +3101,16 @@
         <v>7</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E9" s="9">
         <v>4</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -3150,7 +3150,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="27.6">
@@ -3159,16 +3159,16 @@
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E2" s="9">
         <v>1</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="27.6">
@@ -3179,16 +3179,16 @@
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E3" s="9">
         <v>2</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="27.6">
@@ -3199,16 +3199,16 @@
         <v>2</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E4" s="9">
         <v>3</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.6">
@@ -3219,16 +3219,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E5" s="9">
         <v>3</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.6">
@@ -3239,16 +3239,16 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E6" s="9">
         <v>3</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.6">
@@ -3259,16 +3259,16 @@
         <v>5</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E7" s="9">
         <v>3</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="27.6">
@@ -3279,16 +3279,16 @@
         <v>6</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E8" s="9">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
repairing bugs on gantt utils
</commit_message>
<xml_diff>
--- a/data/project_tasks.xlsx
+++ b/data/project_tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\WW FILES\Indie Project\gantt-plotter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1183BEC7-1C1E-42C2-AB41-8D656506F61F}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F689B3-3E71-464D-A568-E95D79D35DAE}" xr6:coauthVersionLast="38" xr6:coauthVersionMax="38" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="18084" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="36" windowWidth="15960" windowHeight="18084" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="145">
   <si>
     <t>task_id</t>
   </si>
@@ -456,6 +456,9 @@
   </si>
   <si>
     <t>Construct structural frame</t>
+  </si>
+  <si>
+    <t>deadline</t>
   </si>
 </sst>
 </file>
@@ -2601,16 +2604,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A31EC9A9-AD0A-41E7-A100-17EDC0B19FA0}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="24.19921875" customWidth="1"/>
-    <col min="2" max="2" width="15.3984375" customWidth="1"/>
-    <col min="3" max="3" width="16.69921875" customWidth="1"/>
-    <col min="4" max="4" width="18.796875" customWidth="1"/>
+    <col min="2" max="3" width="15.3984375" customWidth="1"/>
+    <col min="4" max="4" width="16.69921875" customWidth="1"/>
+    <col min="5" max="5" width="18.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="8" t="s">
         <v>85</v>
       </c>
@@ -2618,55 +2621,61 @@
         <v>86</v>
       </c>
       <c r="C1" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" s="11" t="s">
         <v>89</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11"/>
+      <c r="D2" s="12">
         <v>46204</v>
       </c>
-      <c r="D2" s="9">
+      <c r="E2" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" s="11" t="s">
         <v>89</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11"/>
+      <c r="D3" s="12">
         <v>46204</v>
       </c>
-      <c r="D3" s="9">
+      <c r="E3" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" s="11" t="s">
         <v>89</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11"/>
+      <c r="D4" s="12">
         <v>46204</v>
       </c>
-      <c r="D4" s="9">
+      <c r="E4" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>90</v>
       </c>
@@ -2674,37 +2683,40 @@
         <v>88</v>
       </c>
       <c r="C5" s="12">
-        <v>46204</v>
-      </c>
-      <c r="D5" s="9">
+        <v>46235</v>
+      </c>
+      <c r="D5" s="12"/>
+      <c r="E5" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>90</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="12">
-        <v>46204</v>
-      </c>
-      <c r="D6" s="9">
+      <c r="C6" s="12"/>
+      <c r="D6" s="12">
+        <v>46199</v>
+      </c>
+      <c r="E6" s="9">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>90</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="12">
-        <v>46204</v>
-      </c>
-      <c r="D7" s="9">
+      <c r="C7" s="12"/>
+      <c r="D7" s="12">
+        <v>46199</v>
+      </c>
+      <c r="E7" s="9">
         <v>0</v>
       </c>
     </row>

</xml_diff>